<commit_message>
Updated Standings, Box Scores
Data Input to EOD 5/23/26
</commit_message>
<xml_diff>
--- a/2025_2026/Playoffs/Brackets.xlsx
+++ b/2025_2026/Playoffs/Brackets.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\NHLStats\2025_2026\Playoffs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A043C336-6EC7-4B2C-96F1-9BAF76A87790}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2B1DA5E-BDF2-482E-A38C-270B347717DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="1590" windowWidth="38640" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Matchups" sheetId="3" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="553" uniqueCount="98">
   <si>
     <t>Eastern Conference Playoff Teams</t>
   </si>
@@ -314,6 +314,12 @@
   </si>
   <si>
     <t>Golden Knights Lead 3-0</t>
+  </si>
+  <si>
+    <t>Hurricanes Lead 2-1</t>
+  </si>
+  <si>
+    <t>Golden Knights Win Series 4-0</t>
   </si>
 </sst>
 </file>
@@ -692,6 +698,39 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -710,46 +749,13 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1033,19 +1039,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J55"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="31.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="32.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.7109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="31.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.6640625" style="1" customWidth="1"/>
     <col min="4" max="4" width="29" style="1" customWidth="1"/>
-    <col min="5" max="5" width="24.28515625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="26.140625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="37.42578125" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="9.140625" style="1"/>
+    <col min="5" max="5" width="24.33203125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="26.109375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="37.44140625" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1053,7 +1059,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>24</v>
       </c>
@@ -1061,7 +1067,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>25</v>
       </c>
@@ -1069,7 +1075,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>26</v>
       </c>
@@ -1077,7 +1083,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>32</v>
       </c>
@@ -1085,7 +1091,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>33</v>
       </c>
@@ -1093,7 +1099,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>34</v>
       </c>
@@ -1101,7 +1107,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>35</v>
       </c>
@@ -1109,7 +1115,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>36</v>
       </c>
@@ -1117,25 +1123,25 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="11" spans="1:7" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="61" t="s">
+    <row r="10" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="11" spans="1:7" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="59" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="61"/>
-      <c r="C11" s="61" t="s">
+      <c r="B11" s="59"/>
+      <c r="C11" s="59" t="s">
         <v>15</v>
       </c>
-      <c r="D11" s="61"/>
-      <c r="E11" s="61" t="s">
+      <c r="D11" s="59"/>
+      <c r="E11" s="59" t="s">
         <v>16</v>
       </c>
-      <c r="F11" s="61"/>
+      <c r="F11" s="59"/>
       <c r="G11" s="4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A12" s="4" t="s">
         <v>4</v>
       </c>
@@ -1158,22 +1164,22 @@
         <v>19</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="59" t="s">
+    <row r="13" spans="1:7" ht="16.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="60" t="s">
         <v>39</v>
       </c>
-      <c r="B13" s="60"/>
-      <c r="C13" s="59" t="s">
+      <c r="B13" s="61"/>
+      <c r="C13" s="60" t="s">
         <v>41</v>
       </c>
-      <c r="D13" s="60"/>
-      <c r="E13" s="59" t="s">
+      <c r="D13" s="61"/>
+      <c r="E13" s="60" t="s">
         <v>17</v>
       </c>
-      <c r="F13" s="60"/>
+      <c r="F13" s="61"/>
       <c r="G13" s="5"/>
     </row>
-    <row r="14" spans="1:7" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
         <v>25</v>
       </c>
@@ -1192,9 +1198,11 @@
       <c r="F14" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="G14" s="6"/>
-    </row>
-    <row r="15" spans="1:7" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G14" s="6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="6" t="s">
         <v>24</v>
       </c>
@@ -1214,17 +1222,17 @@
         <v>38</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="59" t="s">
+    <row r="16" spans="1:7" ht="16.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="60" t="s">
         <v>40</v>
       </c>
-      <c r="B16" s="60"/>
-      <c r="C16" s="59" t="s">
+      <c r="B16" s="61"/>
+      <c r="C16" s="60" t="s">
         <v>41</v>
       </c>
-      <c r="D16" s="60"/>
-    </row>
-    <row r="17" spans="1:4" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="D16" s="61"/>
+    </row>
+    <row r="17" spans="1:4" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
         <v>36</v>
       </c>
@@ -1238,7 +1246,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="6" t="s">
         <v>32</v>
       </c>
@@ -1252,13 +1260,13 @@
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="59" t="s">
+    <row r="19" spans="1:4" ht="16.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="60" t="s">
         <v>39</v>
       </c>
-      <c r="B19" s="60"/>
-    </row>
-    <row r="20" spans="1:4" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="61"/>
+    </row>
+    <row r="20" spans="1:4" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
         <v>26</v>
       </c>
@@ -1266,7 +1274,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="6" t="s">
         <v>33</v>
       </c>
@@ -1274,13 +1282,13 @@
         <v>37</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="59" t="s">
+    <row r="22" spans="1:4" ht="16.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="60" t="s">
         <v>40</v>
       </c>
-      <c r="B22" s="60"/>
-    </row>
-    <row r="23" spans="1:4" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="61"/>
+    </row>
+    <row r="23" spans="1:4" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
         <v>35</v>
       </c>
@@ -1288,7 +1296,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="6" t="s">
         <v>34</v>
       </c>
@@ -1296,64 +1304,64 @@
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
-    <row r="39" spans="7:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="39" spans="7:10" x14ac:dyDescent="0.3">
       <c r="J39" s="2"/>
     </row>
-    <row r="40" spans="7:10" x14ac:dyDescent="0.25">
+    <row r="40" spans="7:10" x14ac:dyDescent="0.3">
       <c r="J40" s="2"/>
     </row>
-    <row r="41" spans="7:10" x14ac:dyDescent="0.25">
+    <row r="41" spans="7:10" x14ac:dyDescent="0.3">
       <c r="J41" s="2"/>
     </row>
-    <row r="42" spans="7:10" x14ac:dyDescent="0.25">
+    <row r="42" spans="7:10" x14ac:dyDescent="0.3">
       <c r="J42" s="2"/>
     </row>
-    <row r="43" spans="7:10" x14ac:dyDescent="0.25">
+    <row r="43" spans="7:10" x14ac:dyDescent="0.3">
       <c r="J43" s="2"/>
     </row>
-    <row r="44" spans="7:10" x14ac:dyDescent="0.25">
+    <row r="44" spans="7:10" x14ac:dyDescent="0.3">
       <c r="H44" s="2"/>
       <c r="J44" s="2"/>
     </row>
-    <row r="45" spans="7:10" x14ac:dyDescent="0.25">
+    <row r="45" spans="7:10" x14ac:dyDescent="0.3">
       <c r="H45" s="2"/>
       <c r="J45" s="2"/>
     </row>
-    <row r="46" spans="7:10" x14ac:dyDescent="0.25">
+    <row r="46" spans="7:10" x14ac:dyDescent="0.3">
       <c r="G46" s="2"/>
       <c r="H46" s="2"/>
       <c r="J46" s="2"/>
     </row>
-    <row r="48" spans="7:10" x14ac:dyDescent="0.25">
+    <row r="48" spans="7:10" x14ac:dyDescent="0.3">
       <c r="J48" s="2"/>
     </row>
-    <row r="49" spans="7:10" x14ac:dyDescent="0.25">
+    <row r="49" spans="7:10" x14ac:dyDescent="0.3">
       <c r="H49" s="2"/>
       <c r="J49" s="2"/>
     </row>
-    <row r="50" spans="7:10" x14ac:dyDescent="0.25">
+    <row r="50" spans="7:10" x14ac:dyDescent="0.3">
       <c r="J50" s="2"/>
     </row>
-    <row r="51" spans="7:10" x14ac:dyDescent="0.25">
+    <row r="51" spans="7:10" x14ac:dyDescent="0.3">
       <c r="G51" s="2"/>
       <c r="J51" s="2"/>
     </row>
-    <row r="52" spans="7:10" x14ac:dyDescent="0.25">
+    <row r="52" spans="7:10" x14ac:dyDescent="0.3">
       <c r="G52" s="2"/>
       <c r="H52" s="2"/>
       <c r="J52" s="2"/>
     </row>
-    <row r="53" spans="7:10" x14ac:dyDescent="0.25">
+    <row r="53" spans="7:10" x14ac:dyDescent="0.3">
       <c r="G53" s="2"/>
       <c r="J53" s="2"/>
     </row>
-    <row r="54" spans="7:10" x14ac:dyDescent="0.25">
+    <row r="54" spans="7:10" x14ac:dyDescent="0.3">
       <c r="G54" s="2"/>
       <c r="H54" s="2"/>
       <c r="J54" s="2"/>
     </row>
-    <row r="55" spans="7:10" x14ac:dyDescent="0.25">
+    <row r="55" spans="7:10" x14ac:dyDescent="0.3">
       <c r="G55" s="2"/>
       <c r="H55" s="2"/>
       <c r="J55" s="2"/>
@@ -1363,16 +1371,16 @@
     <sortCondition ref="B2:B9"/>
   </sortState>
   <mergeCells count="10">
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="C16:D16"/>
     <mergeCell ref="E11:F11"/>
     <mergeCell ref="E13:F13"/>
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="A13:B13"/>
     <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="C16:D16"/>
   </mergeCells>
   <dataValidations count="16">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C14" xr:uid="{2C3D9587-ABAE-4E3F-8B22-396DF812BF02}">
@@ -1432,170 +1440,170 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:BB49"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="1"/>
-    <col min="2" max="2" width="12.7109375" style="19" customWidth="1"/>
-    <col min="3" max="3" width="28.5703125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="9.140625" style="1"/>
-    <col min="5" max="5" width="22.5703125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="9.140625" style="1"/>
-    <col min="7" max="7" width="30.5703125" style="1" customWidth="1"/>
-    <col min="8" max="13" width="9.140625" style="1"/>
-    <col min="14" max="14" width="14.85546875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="9.109375" style="1"/>
+    <col min="2" max="2" width="12.6640625" style="19" customWidth="1"/>
+    <col min="3" max="3" width="28.5546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="9.109375" style="1"/>
+    <col min="5" max="5" width="22.5546875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="9.109375" style="1"/>
+    <col min="7" max="7" width="30.5546875" style="1" customWidth="1"/>
+    <col min="8" max="13" width="9.109375" style="1"/>
+    <col min="14" max="14" width="14.88671875" style="1" customWidth="1"/>
     <col min="15" max="15" width="26" style="1" customWidth="1"/>
     <col min="16" max="16" width="17" style="1" customWidth="1"/>
-    <col min="17" max="17" width="20.140625" style="1" customWidth="1"/>
-    <col min="18" max="18" width="20.28515625" style="1" customWidth="1"/>
-    <col min="19" max="19" width="24.7109375" style="1" customWidth="1"/>
-    <col min="20" max="20" width="23.42578125" style="1" customWidth="1"/>
-    <col min="21" max="21" width="9.140625" style="1"/>
+    <col min="17" max="17" width="20.109375" style="1" customWidth="1"/>
+    <col min="18" max="18" width="20.33203125" style="1" customWidth="1"/>
+    <col min="19" max="19" width="24.6640625" style="1" customWidth="1"/>
+    <col min="20" max="20" width="23.44140625" style="1" customWidth="1"/>
+    <col min="21" max="21" width="9.109375" style="1"/>
     <col min="22" max="22" width="26" style="1" customWidth="1"/>
-    <col min="23" max="23" width="9.140625" style="1"/>
-    <col min="24" max="24" width="21.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="25" max="28" width="21.42578125" style="1" customWidth="1"/>
-    <col min="29" max="29" width="9.140625" style="1"/>
-    <col min="30" max="30" width="22.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="31" max="32" width="9.140625" style="1"/>
-    <col min="33" max="33" width="23.7109375" style="1" customWidth="1"/>
-    <col min="34" max="34" width="22.85546875" style="1" customWidth="1"/>
-    <col min="35" max="36" width="21.7109375" style="1" customWidth="1"/>
-    <col min="37" max="37" width="22.28515625" style="1" customWidth="1"/>
-    <col min="38" max="38" width="25.85546875" style="1" customWidth="1"/>
-    <col min="39" max="39" width="22.140625" style="1" customWidth="1"/>
-    <col min="40" max="40" width="9.140625" style="1"/>
-    <col min="41" max="41" width="29.42578125" style="1" customWidth="1"/>
-    <col min="42" max="47" width="9.140625" style="1"/>
-    <col min="48" max="48" width="10.28515625" style="1" customWidth="1"/>
-    <col min="49" max="49" width="23.140625" style="1" customWidth="1"/>
-    <col min="50" max="50" width="9.140625" style="1"/>
-    <col min="51" max="51" width="23.140625" style="1" customWidth="1"/>
-    <col min="52" max="52" width="9.140625" style="1"/>
-    <col min="53" max="53" width="29.28515625" style="1" customWidth="1"/>
-    <col min="54" max="16384" width="9.140625" style="1"/>
+    <col min="23" max="23" width="9.109375" style="1"/>
+    <col min="24" max="24" width="21.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="25" max="28" width="21.44140625" style="1" customWidth="1"/>
+    <col min="29" max="29" width="9.109375" style="1"/>
+    <col min="30" max="30" width="22.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="31" max="32" width="9.109375" style="1"/>
+    <col min="33" max="33" width="23.6640625" style="1" customWidth="1"/>
+    <col min="34" max="34" width="22.88671875" style="1" customWidth="1"/>
+    <col min="35" max="36" width="21.6640625" style="1" customWidth="1"/>
+    <col min="37" max="37" width="22.33203125" style="1" customWidth="1"/>
+    <col min="38" max="38" width="29.21875" style="1" customWidth="1"/>
+    <col min="39" max="39" width="22.109375" style="1" customWidth="1"/>
+    <col min="40" max="40" width="9.109375" style="1"/>
+    <col min="41" max="41" width="29.44140625" style="1" customWidth="1"/>
+    <col min="42" max="47" width="9.109375" style="1"/>
+    <col min="48" max="48" width="10.33203125" style="1" customWidth="1"/>
+    <col min="49" max="49" width="23.109375" style="1" customWidth="1"/>
+    <col min="50" max="50" width="9.109375" style="1"/>
+    <col min="51" max="51" width="23.109375" style="1" customWidth="1"/>
+    <col min="52" max="52" width="9.109375" style="1"/>
+    <col min="53" max="53" width="29.33203125" style="1" customWidth="1"/>
+    <col min="54" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:54" ht="27.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="51" t="s">
+    <row r="1" spans="1:54" ht="27" thickTop="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" s="50" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="52"/>
-      <c r="C1" s="52"/>
-      <c r="D1" s="52"/>
-      <c r="E1" s="52"/>
-      <c r="F1" s="52"/>
-      <c r="G1" s="52"/>
-      <c r="H1" s="52"/>
-      <c r="I1" s="52"/>
-      <c r="J1" s="52"/>
-      <c r="K1" s="52"/>
-      <c r="L1" s="52"/>
-      <c r="M1" s="52"/>
-      <c r="N1" s="52"/>
-      <c r="O1" s="52"/>
-      <c r="P1" s="52"/>
-      <c r="Q1" s="52"/>
-      <c r="R1" s="52"/>
-      <c r="S1" s="52"/>
-      <c r="T1" s="52"/>
-      <c r="U1" s="53"/>
-      <c r="Z1" s="51" t="s">
+      <c r="B1" s="51"/>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
+      <c r="E1" s="51"/>
+      <c r="F1" s="51"/>
+      <c r="G1" s="51"/>
+      <c r="H1" s="51"/>
+      <c r="I1" s="51"/>
+      <c r="J1" s="51"/>
+      <c r="K1" s="51"/>
+      <c r="L1" s="51"/>
+      <c r="M1" s="51"/>
+      <c r="N1" s="51"/>
+      <c r="O1" s="51"/>
+      <c r="P1" s="51"/>
+      <c r="Q1" s="51"/>
+      <c r="R1" s="51"/>
+      <c r="S1" s="51"/>
+      <c r="T1" s="51"/>
+      <c r="U1" s="52"/>
+      <c r="Z1" s="50" t="s">
         <v>21</v>
       </c>
-      <c r="AA1" s="52"/>
-      <c r="AB1" s="53"/>
-      <c r="AF1" s="51" t="s">
+      <c r="AA1" s="51"/>
+      <c r="AB1" s="52"/>
+      <c r="AF1" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="AG1" s="52"/>
-      <c r="AH1" s="52"/>
-      <c r="AI1" s="52"/>
-      <c r="AJ1" s="52"/>
-      <c r="AK1" s="52"/>
-      <c r="AL1" s="52"/>
-      <c r="AM1" s="52"/>
-      <c r="AN1" s="52"/>
-      <c r="AO1" s="52"/>
-      <c r="AP1" s="52"/>
-      <c r="AQ1" s="52"/>
-      <c r="AR1" s="52"/>
-      <c r="AS1" s="52"/>
-      <c r="AT1" s="52"/>
-      <c r="AU1" s="52"/>
-      <c r="AV1" s="52"/>
-      <c r="AW1" s="52"/>
-      <c r="AX1" s="52"/>
-      <c r="AY1" s="52"/>
-      <c r="AZ1" s="52"/>
-      <c r="BA1" s="53"/>
-    </row>
-    <row r="2" spans="1:54" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="55" t="s">
+      <c r="AG1" s="51"/>
+      <c r="AH1" s="51"/>
+      <c r="AI1" s="51"/>
+      <c r="AJ1" s="51"/>
+      <c r="AK1" s="51"/>
+      <c r="AL1" s="51"/>
+      <c r="AM1" s="51"/>
+      <c r="AN1" s="51"/>
+      <c r="AO1" s="51"/>
+      <c r="AP1" s="51"/>
+      <c r="AQ1" s="51"/>
+      <c r="AR1" s="51"/>
+      <c r="AS1" s="51"/>
+      <c r="AT1" s="51"/>
+      <c r="AU1" s="51"/>
+      <c r="AV1" s="51"/>
+      <c r="AW1" s="51"/>
+      <c r="AX1" s="51"/>
+      <c r="AY1" s="51"/>
+      <c r="AZ1" s="51"/>
+      <c r="BA1" s="52"/>
+    </row>
+    <row r="2" spans="1:54" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="46" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="56"/>
-      <c r="C2" s="56"/>
-      <c r="D2" s="56"/>
-      <c r="E2" s="56"/>
-      <c r="F2" s="56"/>
-      <c r="G2" s="57"/>
-      <c r="M2" s="55" t="s">
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
+      <c r="G2" s="48"/>
+      <c r="M2" s="46" t="s">
         <v>20</v>
       </c>
-      <c r="N2" s="56"/>
-      <c r="O2" s="56"/>
-      <c r="P2" s="56"/>
-      <c r="Q2" s="56"/>
-      <c r="R2" s="57"/>
-      <c r="AI2" s="55" t="s">
+      <c r="N2" s="47"/>
+      <c r="O2" s="47"/>
+      <c r="P2" s="47"/>
+      <c r="Q2" s="47"/>
+      <c r="R2" s="48"/>
+      <c r="AI2" s="46" t="s">
         <v>20</v>
       </c>
-      <c r="AJ2" s="56"/>
-      <c r="AK2" s="56"/>
-      <c r="AL2" s="56"/>
-      <c r="AM2" s="56"/>
-      <c r="AN2" s="56"/>
-      <c r="AO2" s="57"/>
-      <c r="AU2" s="55" t="s">
+      <c r="AJ2" s="47"/>
+      <c r="AK2" s="47"/>
+      <c r="AL2" s="47"/>
+      <c r="AM2" s="47"/>
+      <c r="AN2" s="47"/>
+      <c r="AO2" s="48"/>
+      <c r="AU2" s="46" t="s">
         <v>6</v>
       </c>
-      <c r="AV2" s="56"/>
-      <c r="AW2" s="56"/>
-      <c r="AX2" s="56"/>
-      <c r="AY2" s="56"/>
-      <c r="AZ2" s="56"/>
-      <c r="BA2" s="57"/>
-    </row>
-    <row r="3" spans="1:54" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="49" t="s">
+      <c r="AV2" s="47"/>
+      <c r="AW2" s="47"/>
+      <c r="AX2" s="47"/>
+      <c r="AY2" s="47"/>
+      <c r="AZ2" s="47"/>
+      <c r="BA2" s="48"/>
+    </row>
+    <row r="3" spans="1:54" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="42" t="s">
         <v>42</v>
       </c>
-      <c r="B3" s="49"/>
-      <c r="C3" s="49"/>
-      <c r="D3" s="49"/>
-      <c r="E3" s="49"/>
-      <c r="F3" s="49"/>
-      <c r="G3" s="49"/>
-      <c r="AI3" s="42" t="s">
+      <c r="B3" s="42"/>
+      <c r="C3" s="42"/>
+      <c r="D3" s="42"/>
+      <c r="E3" s="42"/>
+      <c r="F3" s="42"/>
+      <c r="G3" s="42"/>
+      <c r="AI3" s="53" t="s">
         <v>44</v>
       </c>
-      <c r="AJ3" s="43"/>
-      <c r="AK3" s="43"/>
-      <c r="AL3" s="43"/>
-      <c r="AM3" s="43"/>
-      <c r="AN3" s="43"/>
-      <c r="AO3" s="44"/>
-      <c r="AU3" s="49" t="s">
+      <c r="AJ3" s="54"/>
+      <c r="AK3" s="54"/>
+      <c r="AL3" s="54"/>
+      <c r="AM3" s="54"/>
+      <c r="AN3" s="54"/>
+      <c r="AO3" s="55"/>
+      <c r="AU3" s="42" t="s">
         <v>42</v>
       </c>
-      <c r="AV3" s="49"/>
-      <c r="AW3" s="49"/>
-      <c r="AX3" s="49"/>
-      <c r="AY3" s="49"/>
-      <c r="AZ3" s="49"/>
-      <c r="BA3" s="49"/>
-    </row>
-    <row r="4" spans="1:54" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AV3" s="42"/>
+      <c r="AW3" s="42"/>
+      <c r="AX3" s="42"/>
+      <c r="AY3" s="42"/>
+      <c r="AZ3" s="42"/>
+      <c r="BA3" s="42"/>
+    </row>
+    <row r="4" spans="1:54" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -1617,15 +1625,15 @@
       <c r="G4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="M4" s="42" t="s">
+      <c r="M4" s="53" t="s">
         <v>44</v>
       </c>
-      <c r="N4" s="43"/>
-      <c r="O4" s="43"/>
-      <c r="P4" s="43"/>
-      <c r="Q4" s="43"/>
-      <c r="R4" s="43"/>
-      <c r="S4" s="44"/>
+      <c r="N4" s="54"/>
+      <c r="O4" s="54"/>
+      <c r="P4" s="54"/>
+      <c r="Q4" s="54"/>
+      <c r="R4" s="54"/>
+      <c r="S4" s="55"/>
       <c r="AI4" s="3" t="s">
         <v>2</v>
       </c>
@@ -1669,7 +1677,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:54" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:54" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="7">
         <v>1</v>
       </c>
@@ -1755,7 +1763,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="6" spans="1:54" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:54" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A6" s="8">
         <v>2</v>
       </c>
@@ -1844,7 +1852,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="7" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:54" x14ac:dyDescent="0.3">
       <c r="A7" s="8">
         <v>3</v>
       </c>
@@ -1930,7 +1938,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="8" spans="1:54" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:54" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A8" s="8">
         <v>4</v>
       </c>
@@ -1952,11 +1960,11 @@
       <c r="G8" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="I8" s="50" t="s">
+      <c r="I8" s="43" t="s">
         <v>25</v>
       </c>
-      <c r="J8" s="50"/>
-      <c r="K8" s="50"/>
+      <c r="J8" s="43"/>
+      <c r="K8" s="43"/>
       <c r="M8" s="8">
         <v>3</v>
       </c>
@@ -1999,11 +2007,11 @@
       <c r="AO8" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="AQ8" s="50" t="s">
+      <c r="AQ8" s="43" t="s">
         <v>27</v>
       </c>
-      <c r="AR8" s="50"/>
-      <c r="AS8" s="50"/>
+      <c r="AR8" s="43"/>
+      <c r="AS8" s="43"/>
       <c r="AU8" s="38">
         <v>4</v>
       </c>
@@ -2026,7 +2034,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="9" spans="1:54" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:54" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
         <v>11</v>
       </c>
@@ -2116,7 +2124,7 @@
       <c r="AZ9" s="13"/>
       <c r="BA9" s="32"/>
     </row>
-    <row r="10" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:54" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
         <v>10</v>
       </c>
@@ -2192,7 +2200,7 @@
       <c r="AZ10" s="13"/>
       <c r="BA10" s="16"/>
     </row>
-    <row r="11" spans="1:54" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:54" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>12</v>
       </c>
@@ -2262,16 +2270,16 @@
       <c r="AZ11" s="15"/>
       <c r="BA11" s="6"/>
     </row>
-    <row r="12" spans="1:54" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="49" t="s">
+    <row r="12" spans="1:54" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="49"/>
-      <c r="C12" s="49"/>
-      <c r="D12" s="49"/>
-      <c r="E12" s="49"/>
-      <c r="F12" s="49"/>
-      <c r="G12" s="49"/>
+      <c r="B12" s="42"/>
+      <c r="C12" s="42"/>
+      <c r="D12" s="42"/>
+      <c r="E12" s="42"/>
+      <c r="F12" s="42"/>
+      <c r="G12" s="42"/>
       <c r="L12" s="12"/>
       <c r="M12" s="8" t="s">
         <v>12</v>
@@ -2297,71 +2305,71 @@
       <c r="T12" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="AI12" s="49" t="s">
+      <c r="AI12" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="AJ12" s="49"/>
-      <c r="AK12" s="49"/>
-      <c r="AL12" s="49"/>
-      <c r="AM12" s="49"/>
-      <c r="AN12" s="49"/>
-      <c r="AO12" s="49"/>
+      <c r="AJ12" s="42"/>
+      <c r="AK12" s="42"/>
+      <c r="AL12" s="42"/>
+      <c r="AM12" s="42"/>
+      <c r="AN12" s="42"/>
+      <c r="AO12" s="42"/>
       <c r="AQ12" s="12"/>
-      <c r="AU12" s="49" t="s">
+      <c r="AU12" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="AV12" s="49"/>
-      <c r="AW12" s="49"/>
-      <c r="AX12" s="49"/>
-      <c r="AY12" s="49"/>
-      <c r="AZ12" s="49"/>
-      <c r="BA12" s="49"/>
-    </row>
-    <row r="13" spans="1:54" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AV12" s="42"/>
+      <c r="AW12" s="42"/>
+      <c r="AX12" s="42"/>
+      <c r="AY12" s="42"/>
+      <c r="AZ12" s="42"/>
+      <c r="BA12" s="42"/>
+    </row>
+    <row r="13" spans="1:54" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="L13" s="12"/>
-      <c r="M13" s="42" t="s">
+      <c r="M13" s="53" t="s">
         <v>13</v>
       </c>
-      <c r="N13" s="43"/>
-      <c r="O13" s="43"/>
-      <c r="P13" s="43"/>
-      <c r="Q13" s="43"/>
-      <c r="R13" s="43"/>
-      <c r="S13" s="44"/>
+      <c r="N13" s="54"/>
+      <c r="O13" s="54"/>
+      <c r="P13" s="54"/>
+      <c r="Q13" s="54"/>
+      <c r="R13" s="54"/>
+      <c r="S13" s="55"/>
       <c r="AQ13" s="12"/>
     </row>
-    <row r="14" spans="1:54" ht="22.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A14" s="48" t="s">
+    <row r="14" spans="1:54" ht="22.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A14" s="45" t="s">
         <v>43</v>
       </c>
-      <c r="B14" s="48"/>
-      <c r="C14" s="48"/>
-      <c r="D14" s="48"/>
-      <c r="E14" s="48"/>
-      <c r="F14" s="48"/>
-      <c r="G14" s="48"/>
-      <c r="L14" s="54" t="s">
+      <c r="B14" s="45"/>
+      <c r="C14" s="45"/>
+      <c r="D14" s="45"/>
+      <c r="E14" s="45"/>
+      <c r="F14" s="45"/>
+      <c r="G14" s="45"/>
+      <c r="L14" s="44" t="s">
         <v>32</v>
       </c>
-      <c r="M14" s="50"/>
-      <c r="N14" s="50"/>
-      <c r="AN14" s="50" t="s">
+      <c r="M14" s="43"/>
+      <c r="N14" s="43"/>
+      <c r="AN14" s="43" t="s">
         <v>27</v>
       </c>
-      <c r="AO14" s="50"/>
-      <c r="AP14" s="50"/>
+      <c r="AO14" s="43"/>
+      <c r="AP14" s="43"/>
       <c r="AQ14" s="12"/>
-      <c r="AU14" s="48" t="s">
+      <c r="AU14" s="45" t="s">
         <v>43</v>
       </c>
-      <c r="AV14" s="48"/>
-      <c r="AW14" s="48"/>
-      <c r="AX14" s="48"/>
-      <c r="AY14" s="48"/>
-      <c r="AZ14" s="48"/>
-      <c r="BA14" s="48"/>
-    </row>
-    <row r="15" spans="1:54" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AV14" s="45"/>
+      <c r="AW14" s="45"/>
+      <c r="AX14" s="45"/>
+      <c r="AY14" s="45"/>
+      <c r="AZ14" s="45"/>
+      <c r="BA14" s="45"/>
+    </row>
+    <row r="15" spans="1:54" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
         <v>2</v>
       </c>
@@ -2409,7 +2417,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="16" spans="1:54" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:54" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A16" s="7">
         <v>1</v>
       </c>
@@ -2460,7 +2468,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="17" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:54" x14ac:dyDescent="0.3">
       <c r="A17" s="8">
         <v>2</v>
       </c>
@@ -2511,7 +2519,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="18" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:54" x14ac:dyDescent="0.3">
       <c r="A18" s="8">
         <v>3</v>
       </c>
@@ -2565,7 +2573,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="19" spans="1:54" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:54" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A19" s="8">
         <v>4</v>
       </c>
@@ -2587,19 +2595,19 @@
       <c r="G19" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="I19" s="50" t="s">
+      <c r="I19" s="43" t="s">
         <v>32</v>
       </c>
-      <c r="J19" s="50"/>
-      <c r="K19" s="50"/>
+      <c r="J19" s="43"/>
+      <c r="K19" s="43"/>
       <c r="L19" s="12"/>
       <c r="O19" s="12"/>
       <c r="AN19" s="12"/>
-      <c r="AQ19" s="54" t="s">
+      <c r="AQ19" s="44" t="s">
         <v>31</v>
       </c>
-      <c r="AR19" s="50"/>
-      <c r="AS19" s="50"/>
+      <c r="AR19" s="43"/>
+      <c r="AS19" s="43"/>
       <c r="AU19" s="38">
         <v>4</v>
       </c>
@@ -2625,7 +2633,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="20" spans="1:54" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:54" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
         <v>11</v>
       </c>
@@ -2671,7 +2679,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="21" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:54" x14ac:dyDescent="0.3">
       <c r="A21" s="8" t="s">
         <v>10</v>
       </c>
@@ -2720,7 +2728,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="22" spans="1:54" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:54" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="9" t="s">
         <v>12</v>
       </c>
@@ -2760,55 +2768,55 @@
       <c r="AZ22" s="15"/>
       <c r="BA22" s="6"/>
     </row>
-    <row r="23" spans="1:54" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="49" t="s">
+    <row r="23" spans="1:54" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="B23" s="49"/>
-      <c r="C23" s="49"/>
-      <c r="D23" s="49"/>
-      <c r="E23" s="49"/>
-      <c r="F23" s="49"/>
-      <c r="G23" s="49"/>
+      <c r="B23" s="42"/>
+      <c r="C23" s="42"/>
+      <c r="D23" s="42"/>
+      <c r="E23" s="42"/>
+      <c r="F23" s="42"/>
+      <c r="G23" s="42"/>
       <c r="O23" s="12"/>
       <c r="AN23" s="12"/>
-      <c r="AU23" s="49" t="s">
+      <c r="AU23" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="AV23" s="49"/>
-      <c r="AW23" s="49"/>
-      <c r="AX23" s="49"/>
-      <c r="AY23" s="49"/>
-      <c r="AZ23" s="49"/>
-      <c r="BA23" s="49"/>
-    </row>
-    <row r="24" spans="1:54" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AV23" s="42"/>
+      <c r="AW23" s="42"/>
+      <c r="AX23" s="42"/>
+      <c r="AY23" s="42"/>
+      <c r="AZ23" s="42"/>
+      <c r="BA23" s="42"/>
+    </row>
+    <row r="24" spans="1:54" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="O24" s="12"/>
       <c r="AN24" s="12"/>
     </row>
-    <row r="25" spans="1:54" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="49" t="s">
+    <row r="25" spans="1:54" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="42" t="s">
         <v>42</v>
       </c>
-      <c r="B25" s="49"/>
-      <c r="C25" s="49"/>
-      <c r="D25" s="49"/>
-      <c r="E25" s="49"/>
-      <c r="F25" s="49"/>
-      <c r="G25" s="49"/>
+      <c r="B25" s="42"/>
+      <c r="C25" s="42"/>
+      <c r="D25" s="42"/>
+      <c r="E25" s="42"/>
+      <c r="F25" s="42"/>
+      <c r="G25" s="42"/>
       <c r="O25" s="12"/>
       <c r="AN25" s="12"/>
-      <c r="AU25" s="49" t="s">
+      <c r="AU25" s="42" t="s">
         <v>42</v>
       </c>
-      <c r="AV25" s="49"/>
-      <c r="AW25" s="49"/>
-      <c r="AX25" s="49"/>
-      <c r="AY25" s="49"/>
-      <c r="AZ25" s="49"/>
-      <c r="BA25" s="49"/>
-    </row>
-    <row r="26" spans="1:54" ht="22.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="AV25" s="42"/>
+      <c r="AW25" s="42"/>
+      <c r="AX25" s="42"/>
+      <c r="AY25" s="42"/>
+      <c r="AZ25" s="42"/>
+      <c r="BA25" s="42"/>
+    </row>
+    <row r="26" spans="1:54" ht="22.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A26" s="20" t="s">
         <v>2</v>
       </c>
@@ -2830,24 +2838,26 @@
       <c r="G26" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="O26" s="54"/>
-      <c r="P26" s="50"/>
-      <c r="Q26" s="50"/>
-      <c r="R26" s="50"/>
-      <c r="S26" s="50"/>
-      <c r="T26" s="50"/>
-      <c r="U26" s="50"/>
-      <c r="V26" s="50"/>
-      <c r="W26" s="50"/>
-      <c r="AE26" s="50"/>
-      <c r="AF26" s="50"/>
-      <c r="AG26" s="50"/>
-      <c r="AH26" s="50"/>
-      <c r="AI26" s="50"/>
-      <c r="AJ26" s="50"/>
-      <c r="AK26" s="50"/>
-      <c r="AL26" s="50"/>
-      <c r="AM26" s="58"/>
+      <c r="O26" s="44"/>
+      <c r="P26" s="43"/>
+      <c r="Q26" s="43"/>
+      <c r="R26" s="43"/>
+      <c r="S26" s="43"/>
+      <c r="T26" s="43"/>
+      <c r="U26" s="43"/>
+      <c r="V26" s="43"/>
+      <c r="W26" s="43"/>
+      <c r="AE26" s="43" t="s">
+        <v>38</v>
+      </c>
+      <c r="AF26" s="43"/>
+      <c r="AG26" s="43"/>
+      <c r="AH26" s="43"/>
+      <c r="AI26" s="43"/>
+      <c r="AJ26" s="43"/>
+      <c r="AK26" s="43"/>
+      <c r="AL26" s="43"/>
+      <c r="AM26" s="49"/>
       <c r="AU26" s="20" t="s">
         <v>2</v>
       </c>
@@ -2870,7 +2880,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="27" spans="1:54" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:54" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="7">
         <v>1</v>
       </c>
@@ -2918,7 +2928,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="28" spans="1:54" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:54" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="8">
         <v>2</v>
       </c>
@@ -2944,26 +2954,26 @@
         <v>54</v>
       </c>
       <c r="O28" s="12"/>
-      <c r="P28" s="42" t="s">
+      <c r="P28" s="53" t="s">
         <v>16</v>
       </c>
-      <c r="Q28" s="43"/>
-      <c r="R28" s="43"/>
-      <c r="S28" s="43"/>
-      <c r="T28" s="43"/>
-      <c r="U28" s="43"/>
-      <c r="V28" s="44"/>
+      <c r="Q28" s="54"/>
+      <c r="R28" s="54"/>
+      <c r="S28" s="54"/>
+      <c r="T28" s="54"/>
+      <c r="U28" s="54"/>
+      <c r="V28" s="55"/>
       <c r="X28" s="12"/>
       <c r="AD28" s="13"/>
-      <c r="AF28" s="49" t="s">
+      <c r="AF28" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="AG28" s="49"/>
-      <c r="AH28" s="49"/>
-      <c r="AI28" s="49"/>
-      <c r="AJ28" s="49"/>
-      <c r="AK28" s="49"/>
-      <c r="AL28" s="49"/>
+      <c r="AG28" s="42"/>
+      <c r="AH28" s="42"/>
+      <c r="AI28" s="42"/>
+      <c r="AJ28" s="42"/>
+      <c r="AK28" s="42"/>
+      <c r="AL28" s="42"/>
       <c r="AN28" s="12"/>
       <c r="AU28" s="8">
         <v>2</v>
@@ -2987,7 +2997,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="29" spans="1:54" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:54" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="8">
         <v>3</v>
       </c>
@@ -3077,7 +3087,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="30" spans="1:54" ht="22.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:54" ht="22.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A30" s="8">
         <v>4</v>
       </c>
@@ -3099,11 +3109,11 @@
       <c r="G30" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="I30" s="50" t="s">
+      <c r="I30" s="43" t="s">
         <v>26</v>
       </c>
-      <c r="J30" s="50"/>
-      <c r="K30" s="50"/>
+      <c r="J30" s="43"/>
+      <c r="K30" s="43"/>
       <c r="O30" s="12"/>
       <c r="P30" s="7">
         <v>1</v>
@@ -3150,11 +3160,11 @@
         <v>52</v>
       </c>
       <c r="AN30" s="12"/>
-      <c r="AQ30" s="50" t="s">
+      <c r="AQ30" s="43" t="s">
         <v>38</v>
       </c>
-      <c r="AR30" s="50"/>
-      <c r="AS30" s="50"/>
+      <c r="AR30" s="43"/>
+      <c r="AS30" s="43"/>
       <c r="AU30" s="38">
         <v>4</v>
       </c>
@@ -3180,7 +3190,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="31" spans="1:54" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:54" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A31" s="8" t="s">
         <v>11</v>
       </c>
@@ -3271,7 +3281,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="32" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:54" x14ac:dyDescent="0.3">
       <c r="A32" s="8" t="s">
         <v>10</v>
       </c>
@@ -3298,12 +3308,21 @@
       <c r="R32" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="S32" s="13"/>
+      <c r="S32" s="13">
+        <v>3</v>
+      </c>
       <c r="T32" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="U32" s="13"/>
-      <c r="V32" s="16"/>
+      <c r="U32" s="13">
+        <v>2</v>
+      </c>
+      <c r="V32" s="16" t="s">
+        <v>96</v>
+      </c>
+      <c r="W32" s="1" t="s">
+        <v>49</v>
+      </c>
       <c r="X32" s="12"/>
       <c r="AD32" s="13"/>
       <c r="AF32" s="8">
@@ -3351,7 +3370,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="33" spans="1:54" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:54" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A33" s="9" t="s">
         <v>12</v>
       </c>
@@ -3395,12 +3414,18 @@
       <c r="AH33" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="AI33" s="13"/>
+      <c r="AI33" s="13">
+        <v>1</v>
+      </c>
       <c r="AJ33" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="AK33" s="13"/>
-      <c r="AL33" s="16"/>
+      <c r="AK33" s="13">
+        <v>2</v>
+      </c>
+      <c r="AL33" s="16" t="s">
+        <v>97</v>
+      </c>
       <c r="AN33" s="12"/>
       <c r="AQ33" s="12"/>
       <c r="AU33" s="9" t="s">
@@ -3419,16 +3444,16 @@
       <c r="AZ33" s="15"/>
       <c r="BA33" s="6"/>
     </row>
-    <row r="34" spans="1:54" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="49" t="s">
+    <row r="34" spans="1:54" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="B34" s="49"/>
-      <c r="C34" s="49"/>
-      <c r="D34" s="49"/>
-      <c r="E34" s="49"/>
-      <c r="F34" s="49"/>
-      <c r="G34" s="49"/>
+      <c r="B34" s="42"/>
+      <c r="C34" s="42"/>
+      <c r="D34" s="42"/>
+      <c r="E34" s="42"/>
+      <c r="F34" s="42"/>
+      <c r="G34" s="42"/>
       <c r="L34" s="12"/>
       <c r="O34" s="12"/>
       <c r="P34" s="8" t="s">
@@ -3465,17 +3490,17 @@
       <c r="AL34" s="16"/>
       <c r="AN34" s="12"/>
       <c r="AQ34" s="12"/>
-      <c r="AU34" s="49" t="s">
+      <c r="AU34" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="AV34" s="49"/>
-      <c r="AW34" s="49"/>
-      <c r="AX34" s="49"/>
-      <c r="AY34" s="49"/>
-      <c r="AZ34" s="49"/>
-      <c r="BA34" s="49"/>
-    </row>
-    <row r="35" spans="1:54" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AV34" s="42"/>
+      <c r="AW34" s="42"/>
+      <c r="AX34" s="42"/>
+      <c r="AY34" s="42"/>
+      <c r="AZ34" s="42"/>
+      <c r="BA34" s="42"/>
+    </row>
+    <row r="35" spans="1:54" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="L35" s="12"/>
       <c r="O35" s="12"/>
       <c r="P35" s="8" t="s">
@@ -3513,21 +3538,21 @@
       <c r="AN35" s="12"/>
       <c r="AQ35" s="12"/>
     </row>
-    <row r="36" spans="1:54" ht="22.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A36" s="48" t="s">
+    <row r="36" spans="1:54" ht="22.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A36" s="45" t="s">
         <v>43</v>
       </c>
-      <c r="B36" s="48"/>
-      <c r="C36" s="48"/>
-      <c r="D36" s="48"/>
-      <c r="E36" s="48"/>
-      <c r="F36" s="48"/>
-      <c r="G36" s="48"/>
-      <c r="L36" s="54" t="s">
+      <c r="B36" s="45"/>
+      <c r="C36" s="45"/>
+      <c r="D36" s="45"/>
+      <c r="E36" s="45"/>
+      <c r="F36" s="45"/>
+      <c r="G36" s="45"/>
+      <c r="L36" s="44" t="s">
         <v>26</v>
       </c>
-      <c r="M36" s="50"/>
-      <c r="N36" s="50"/>
+      <c r="M36" s="43"/>
+      <c r="N36" s="43"/>
       <c r="O36" s="12"/>
       <c r="P36" s="8" t="s">
         <v>12</v>
@@ -3561,23 +3586,23 @@
       </c>
       <c r="AK36" s="36"/>
       <c r="AL36" s="37"/>
-      <c r="AN36" s="54" t="s">
+      <c r="AN36" s="44" t="s">
         <v>38</v>
       </c>
-      <c r="AO36" s="50"/>
-      <c r="AP36" s="50"/>
+      <c r="AO36" s="43"/>
+      <c r="AP36" s="43"/>
       <c r="AQ36" s="12"/>
-      <c r="AU36" s="48" t="s">
+      <c r="AU36" s="45" t="s">
         <v>43</v>
       </c>
-      <c r="AV36" s="48"/>
-      <c r="AW36" s="48"/>
-      <c r="AX36" s="48"/>
-      <c r="AY36" s="48"/>
-      <c r="AZ36" s="48"/>
-      <c r="BA36" s="48"/>
-    </row>
-    <row r="37" spans="1:54" ht="22.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="AV36" s="45"/>
+      <c r="AW36" s="45"/>
+      <c r="AX36" s="45"/>
+      <c r="AY36" s="45"/>
+      <c r="AZ36" s="45"/>
+      <c r="BA36" s="45"/>
+    </row>
+    <row r="37" spans="1:54" ht="22.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A37" s="20" t="s">
         <v>2</v>
       </c>
@@ -3600,31 +3625,31 @@
         <v>9</v>
       </c>
       <c r="L37" s="12"/>
-      <c r="P37" s="45" t="s">
+      <c r="P37" s="56" t="s">
         <v>13</v>
       </c>
-      <c r="Q37" s="46"/>
-      <c r="R37" s="46"/>
-      <c r="S37" s="46"/>
-      <c r="T37" s="46"/>
-      <c r="U37" s="46"/>
-      <c r="V37" s="47"/>
-      <c r="X37" s="54"/>
-      <c r="Y37" s="50"/>
-      <c r="Z37" s="50"/>
-      <c r="AA37" s="50"/>
-      <c r="AB37" s="50"/>
-      <c r="AC37" s="50"/>
-      <c r="AD37" s="58"/>
-      <c r="AF37" s="49" t="s">
+      <c r="Q37" s="57"/>
+      <c r="R37" s="57"/>
+      <c r="S37" s="57"/>
+      <c r="T37" s="57"/>
+      <c r="U37" s="57"/>
+      <c r="V37" s="58"/>
+      <c r="X37" s="44"/>
+      <c r="Y37" s="43"/>
+      <c r="Z37" s="43"/>
+      <c r="AA37" s="43"/>
+      <c r="AB37" s="43"/>
+      <c r="AC37" s="43"/>
+      <c r="AD37" s="49"/>
+      <c r="AF37" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="AG37" s="49"/>
-      <c r="AH37" s="49"/>
-      <c r="AI37" s="49"/>
-      <c r="AJ37" s="49"/>
-      <c r="AK37" s="49"/>
-      <c r="AL37" s="49"/>
+      <c r="AG37" s="42"/>
+      <c r="AH37" s="42"/>
+      <c r="AI37" s="42"/>
+      <c r="AJ37" s="42"/>
+      <c r="AK37" s="42"/>
+      <c r="AL37" s="42"/>
       <c r="AQ37" s="12"/>
       <c r="AU37" s="3" t="s">
         <v>2</v>
@@ -3648,7 +3673,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="38" spans="1:54" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:54" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A38" s="7">
         <v>1</v>
       </c>
@@ -3694,7 +3719,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="39" spans="1:54" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:54" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A39" s="8">
         <v>2</v>
       </c>
@@ -3717,33 +3742,33 @@
         <v>53</v>
       </c>
       <c r="L39" s="12"/>
-      <c r="M39" s="42" t="s">
+      <c r="M39" s="53" t="s">
         <v>44</v>
       </c>
-      <c r="N39" s="43"/>
-      <c r="O39" s="43"/>
-      <c r="P39" s="43"/>
-      <c r="Q39" s="43"/>
-      <c r="R39" s="43"/>
-      <c r="S39" s="44"/>
-      <c r="X39" s="49" t="s">
+      <c r="N39" s="54"/>
+      <c r="O39" s="54"/>
+      <c r="P39" s="54"/>
+      <c r="Q39" s="54"/>
+      <c r="R39" s="54"/>
+      <c r="S39" s="55"/>
+      <c r="X39" s="42" t="s">
         <v>21</v>
       </c>
-      <c r="Y39" s="49"/>
-      <c r="Z39" s="49"/>
-      <c r="AA39" s="49"/>
-      <c r="AB39" s="49"/>
-      <c r="AC39" s="49"/>
-      <c r="AD39" s="49"/>
-      <c r="AI39" s="42" t="s">
+      <c r="Y39" s="42"/>
+      <c r="Z39" s="42"/>
+      <c r="AA39" s="42"/>
+      <c r="AB39" s="42"/>
+      <c r="AC39" s="42"/>
+      <c r="AD39" s="42"/>
+      <c r="AI39" s="53" t="s">
         <v>44</v>
       </c>
-      <c r="AJ39" s="43"/>
-      <c r="AK39" s="43"/>
-      <c r="AL39" s="43"/>
-      <c r="AM39" s="43"/>
-      <c r="AN39" s="43"/>
-      <c r="AO39" s="44"/>
+      <c r="AJ39" s="54"/>
+      <c r="AK39" s="54"/>
+      <c r="AL39" s="54"/>
+      <c r="AM39" s="54"/>
+      <c r="AN39" s="54"/>
+      <c r="AO39" s="55"/>
       <c r="AQ39" s="12"/>
       <c r="AU39" s="8">
         <v>2</v>
@@ -3767,7 +3792,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="40" spans="1:54" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:54" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A40" s="8">
         <v>3</v>
       </c>
@@ -3876,7 +3901,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="41" spans="1:54" ht="22.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:54" ht="22.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A41" s="8">
         <v>4</v>
       </c>
@@ -3898,11 +3923,11 @@
       <c r="G41" s="16" t="s">
         <v>69</v>
       </c>
-      <c r="I41" s="50" t="s">
+      <c r="I41" s="43" t="s">
         <v>34</v>
       </c>
-      <c r="J41" s="50"/>
-      <c r="K41" s="50"/>
+      <c r="J41" s="43"/>
+      <c r="K41" s="43"/>
       <c r="L41" s="12"/>
       <c r="M41" s="7">
         <v>1</v>
@@ -3955,11 +3980,11 @@
       <c r="AO41" s="25" t="s">
         <v>87</v>
       </c>
-      <c r="AQ41" s="54" t="s">
+      <c r="AQ41" s="44" t="s">
         <v>23</v>
       </c>
-      <c r="AR41" s="50"/>
-      <c r="AS41" s="50"/>
+      <c r="AR41" s="43"/>
+      <c r="AS41" s="43"/>
       <c r="AU41" s="38">
         <v>4</v>
       </c>
@@ -3985,7 +4010,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="42" spans="1:54" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:54" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A42" s="8" t="s">
         <v>11</v>
       </c>
@@ -4080,7 +4105,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="43" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:54" x14ac:dyDescent="0.3">
       <c r="A43" s="8" t="s">
         <v>10</v>
       </c>
@@ -4178,7 +4203,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="44" spans="1:54" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:54" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A44" s="9" t="s">
         <v>12</v>
       </c>
@@ -4264,16 +4289,16 @@
       <c r="AZ44" s="15"/>
       <c r="BA44" s="6"/>
     </row>
-    <row r="45" spans="1:54" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="49" t="s">
+    <row r="45" spans="1:54" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A45" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="B45" s="49"/>
-      <c r="C45" s="49"/>
-      <c r="D45" s="49"/>
-      <c r="E45" s="49"/>
-      <c r="F45" s="49"/>
-      <c r="G45" s="49"/>
+      <c r="B45" s="42"/>
+      <c r="C45" s="42"/>
+      <c r="D45" s="42"/>
+      <c r="E45" s="42"/>
+      <c r="F45" s="42"/>
+      <c r="G45" s="42"/>
       <c r="M45" s="8" t="s">
         <v>11</v>
       </c>
@@ -4322,17 +4347,17 @@
       <c r="AP45" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="AU45" s="49" t="s">
+      <c r="AU45" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="AV45" s="49"/>
-      <c r="AW45" s="49"/>
-      <c r="AX45" s="49"/>
-      <c r="AY45" s="49"/>
-      <c r="AZ45" s="49"/>
-      <c r="BA45" s="49"/>
-    </row>
-    <row r="46" spans="1:54" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="AV45" s="42"/>
+      <c r="AW45" s="42"/>
+      <c r="AX45" s="42"/>
+      <c r="AY45" s="42"/>
+      <c r="AZ45" s="42"/>
+      <c r="BA45" s="42"/>
+    </row>
+    <row r="46" spans="1:54" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="M46" s="8" t="s">
         <v>10</v>
       </c>
@@ -4379,7 +4404,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="47" spans="1:54" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:54" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="M47" s="8" t="s">
         <v>12</v>
       </c>
@@ -4420,50 +4445,62 @@
       <c r="AN47" s="15"/>
       <c r="AO47" s="6"/>
     </row>
-    <row r="48" spans="1:54" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="M48" s="42" t="s">
+    <row r="48" spans="1:54" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="M48" s="53" t="s">
         <v>13</v>
       </c>
-      <c r="N48" s="43"/>
-      <c r="O48" s="43"/>
-      <c r="P48" s="43"/>
-      <c r="Q48" s="43"/>
-      <c r="R48" s="43"/>
-      <c r="S48" s="44"/>
-      <c r="X48" s="49" t="s">
+      <c r="N48" s="54"/>
+      <c r="O48" s="54"/>
+      <c r="P48" s="54"/>
+      <c r="Q48" s="54"/>
+      <c r="R48" s="54"/>
+      <c r="S48" s="55"/>
+      <c r="X48" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="Y48" s="49"/>
-      <c r="Z48" s="49"/>
-      <c r="AA48" s="49"/>
-      <c r="AB48" s="49"/>
-      <c r="AC48" s="49"/>
-      <c r="AD48" s="49"/>
-      <c r="AI48" s="49" t="s">
+      <c r="Y48" s="42"/>
+      <c r="Z48" s="42"/>
+      <c r="AA48" s="42"/>
+      <c r="AB48" s="42"/>
+      <c r="AC48" s="42"/>
+      <c r="AD48" s="42"/>
+      <c r="AI48" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="AJ48" s="49"/>
-      <c r="AK48" s="49"/>
-      <c r="AL48" s="49"/>
-      <c r="AM48" s="49"/>
-      <c r="AN48" s="49"/>
-      <c r="AO48" s="49"/>
-    </row>
-    <row r="49" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+      <c r="AJ48" s="42"/>
+      <c r="AK48" s="42"/>
+      <c r="AL48" s="42"/>
+      <c r="AM48" s="42"/>
+      <c r="AN48" s="42"/>
+      <c r="AO48" s="42"/>
+    </row>
+    <row r="49" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="52">
-    <mergeCell ref="AU45:BA45"/>
-    <mergeCell ref="AF28:AL28"/>
-    <mergeCell ref="AF37:AL37"/>
-    <mergeCell ref="AQ30:AS30"/>
-    <mergeCell ref="AQ41:AS41"/>
-    <mergeCell ref="AU34:BA34"/>
-    <mergeCell ref="AU36:BA36"/>
-    <mergeCell ref="AU2:BA2"/>
-    <mergeCell ref="AU3:BA3"/>
-    <mergeCell ref="AU12:BA12"/>
-    <mergeCell ref="AU14:BA14"/>
-    <mergeCell ref="AU23:BA23"/>
+    <mergeCell ref="M48:S48"/>
+    <mergeCell ref="M39:S39"/>
+    <mergeCell ref="P37:V37"/>
+    <mergeCell ref="P28:V28"/>
+    <mergeCell ref="A36:G36"/>
+    <mergeCell ref="A45:G45"/>
+    <mergeCell ref="I30:K30"/>
+    <mergeCell ref="A34:G34"/>
+    <mergeCell ref="A1:U1"/>
+    <mergeCell ref="O26:W26"/>
+    <mergeCell ref="I41:K41"/>
+    <mergeCell ref="L14:N14"/>
+    <mergeCell ref="L36:N36"/>
+    <mergeCell ref="M2:R2"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="M4:S4"/>
+    <mergeCell ref="M13:S13"/>
+    <mergeCell ref="A12:G12"/>
+    <mergeCell ref="A14:G14"/>
+    <mergeCell ref="A23:G23"/>
+    <mergeCell ref="I8:K8"/>
+    <mergeCell ref="I19:K19"/>
+    <mergeCell ref="A25:G25"/>
     <mergeCell ref="X37:AD37"/>
     <mergeCell ref="AE26:AM26"/>
     <mergeCell ref="Z1:AB1"/>
@@ -4480,30 +4517,18 @@
     <mergeCell ref="AN36:AP36"/>
     <mergeCell ref="AQ8:AS8"/>
     <mergeCell ref="AQ19:AS19"/>
-    <mergeCell ref="A1:U1"/>
-    <mergeCell ref="O26:W26"/>
-    <mergeCell ref="I41:K41"/>
-    <mergeCell ref="L14:N14"/>
-    <mergeCell ref="L36:N36"/>
-    <mergeCell ref="M2:R2"/>
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="M4:S4"/>
-    <mergeCell ref="M13:S13"/>
-    <mergeCell ref="A12:G12"/>
-    <mergeCell ref="A14:G14"/>
-    <mergeCell ref="A23:G23"/>
-    <mergeCell ref="I8:K8"/>
-    <mergeCell ref="I19:K19"/>
-    <mergeCell ref="A25:G25"/>
-    <mergeCell ref="M48:S48"/>
-    <mergeCell ref="M39:S39"/>
-    <mergeCell ref="P37:V37"/>
-    <mergeCell ref="P28:V28"/>
-    <mergeCell ref="A36:G36"/>
-    <mergeCell ref="A45:G45"/>
-    <mergeCell ref="I30:K30"/>
-    <mergeCell ref="A34:G34"/>
+    <mergeCell ref="AU2:BA2"/>
+    <mergeCell ref="AU3:BA3"/>
+    <mergeCell ref="AU12:BA12"/>
+    <mergeCell ref="AU14:BA14"/>
+    <mergeCell ref="AU23:BA23"/>
+    <mergeCell ref="AU45:BA45"/>
+    <mergeCell ref="AF28:AL28"/>
+    <mergeCell ref="AF37:AL37"/>
+    <mergeCell ref="AQ30:AS30"/>
+    <mergeCell ref="AQ41:AS41"/>
+    <mergeCell ref="AU34:BA34"/>
+    <mergeCell ref="AU36:BA36"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>